<commit_message>
Refresh employee meta titles and descriptions in AI optimized Excel
Update columns C–F for all 48 employee story URLs in
lkk_meta_crawl_AI_optimized.xlsx with extracted names, roles, and intro quotes.

Co-authored-by: Terencefong62 <Terencefong62@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/exports/lkk_meta_crawl_AI_optimized.xlsx
+++ b/exports/lkk_meta_crawl_AI_optimized.xlsx
@@ -1337,10 +1337,14 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>adam-ho</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="n"/>
+          <t>Adam Ho | Employee Stories | Lee Kum Kee Corporate</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Adam Ho, IT Manager at Lee Kum Kee. Very often, issues were resolved as a result of discussion and collaboration across teams from different regions.</t>
+        </is>
+      </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
           <t>Adam Ho | Employee Stories | Lee Kum Kee Corporate</t>
@@ -1365,10 +1369,14 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>cheng-chiu-ming</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="n"/>
+          <t>Cheng Chiu Ming (Retired) | Employee Stories | Lee Kum Kee Corporate</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Cheng Chiu Ming (Retired), Manufacturing Manager at Lee Kum Kee. “Corporate culture forms important guiding principles for all staff. We will be working e…</t>
+        </is>
+      </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
           <t>Cheng Chiu Ming (Retired) | Employee Stories | Lee Kum Kee Corporate</t>
@@ -1393,10 +1401,14 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>cheng-wei-yan</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="n"/>
+          <t>Cheng Wei Yan | Employee Stories | Lee Kum Kee Corporate</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Cheng Wei Yan, Assistant Manager at Lee Kum Kee. So far, I perceive the most significant change in my work is that I have taken up more management duties;…</t>
+        </is>
+      </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
           <t>Cheng Wei Yan | Employee Stories | Lee Kum Kee Corporate</t>
@@ -1421,10 +1433,14 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>gong-min</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="n"/>
+          <t>Gong Min | Employee Stories | Lee Kum Kee Corporate</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Gong Min, Finance Manager at Lee Kum Kee. As an Accountant handling the Company’s tax affairs, I have gained a thorough understanding of our corporate cul…</t>
+        </is>
+      </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
           <t>Gong Min | Employee Stories | Lee Kum Kee Corporate</t>
@@ -1449,10 +1465,14 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>jiang-zhi</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="n"/>
+          <t>Jiang Zhi | Employee Stories | Lee Kum Kee Corporate</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Jiang Zhi, Assistant Manager at Lee Kum Kee. I very much admire Lee Kum Kee’s corporate culture and in particular go by the core values of “Pragmatism” an…</t>
+        </is>
+      </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
           <t>Jiang Zhi | Employee Stories | Lee Kum Kee Corporate</t>
@@ -1477,10 +1497,14 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>lau-fung-ying-christine</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="n"/>
+          <t>Christine Lau | Employee Stories | Lee Kum Kee Corporate</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Christine Lau, Senior Business Development Manager at Lee Kum Kee. Our corporate culture emphasizes on “Putting Yourselves in Others’ Shoes” and “Caring A…</t>
+        </is>
+      </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
           <t>Christine Lau | Employee Stories | Lee Kum Kee Corporate</t>
@@ -1505,10 +1529,14 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>mark-butzke</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="n"/>
+          <t>Mark Butzke | Employee Stories | Lee Kum Kee Corporate</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Mark Butzke, Sales Director at Lee Kum Kee. Lee Kum Kee provides the necessary tools for me to grow professionally.</t>
+        </is>
+      </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
           <t>Mark Butzke | Employee Stories | Lee Kum Kee Corporate</t>
@@ -1533,10 +1561,14 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>mauricio-olmedo</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="n"/>
+          <t>Mauricio Olmedo | Employee Stories | Lee Kum Kee Corporate</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Mauricio Olmedo, Production Manager at Lee Kum Kee. I have not only learned a lot about the food industry, production process and regulations, but also th…</t>
+        </is>
+      </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
           <t>Mauricio Olmedo | Employee Stories | Lee Kum Kee Corporate</t>
@@ -1561,10 +1593,14 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>ng-seow-voon-miko</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="n"/>
+          <t>Miko Ng | Employee Stories | Lee Kum Kee Corporate</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Miko Ng, Regional Category Manager, Oyster at Lee Kum Kee. Although I have joined Lee Kum Kee only for a short period of time, I have learned a lot and fo…</t>
+        </is>
+      </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
           <t>Miko Ng | Employee Stories | Lee Kum Kee Corporate</t>
@@ -1589,10 +1625,14 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>ou-yang-tong</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="n"/>
+          <t>Ou Yang Tong | Employee Stories | Lee Kum Kee Corporate</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Ou Yang Tong, Operations Assistant at Lee Kum Kee. Though work was overwhelming and challenging, I gained countless opportunities to sharpen my skills and…</t>
+        </is>
+      </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
           <t>Ou Yang Tong | Employee Stories | Lee Kum Kee Corporate</t>
@@ -1617,10 +1657,14 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>tony-mok</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="n"/>
+          <t>Tony Mok | Employee Stories | Lee Kum Kee Corporate</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Tony Mok, General Manager – Xinhui &amp; Huangpu Plant at Lee Kum Kee. “I started as an officer trainee in the Manufacturing Function. Today, I manage a team…</t>
+        </is>
+      </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
           <t>Tony Mok | Employee Stories | Lee Kum Kee Corporate</t>
@@ -1645,10 +1689,14 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>wei-gang</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="n"/>
+          <t>Wei Gang | Employee Stories | Lee Kum Kee Corporate</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Wei Gang, Associate Regional Sales Director at Lee Kum Kee. '100-1=0' is one of Lee Kum Kee’s corporate cultures that speaks to its constant pursuit of th…</t>
+        </is>
+      </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
           <t>Wei Gang | Employee Stories | Lee Kum Kee Corporate</t>
@@ -1673,10 +1721,14 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>wen-wen</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="n"/>
+          <t>Wen Wen | Employee Stories | Lee Kum Kee Corporate</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Wen Wen, Marketing Manager at Lee Kum Kee. I loved the classic design of its product packaging, which emanates a sense of quality assurance and profession…</t>
+        </is>
+      </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
           <t>Wen Wen | Employee Stories | Lee Kum Kee Corporate</t>
@@ -1701,10 +1753,14 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>wu-zhi-gang-jacky</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="n"/>
+          <t>Jacky Wu | Employee Stories | Lee Kum Kee Corporate</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Jacky Wu, Operation Director at Lee Kum Kee. I believe it is essential for one to keep learning. In addition, we should make use of the strengths of every…</t>
+        </is>
+      </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
           <t>Jacky Wu | Employee Stories | Lee Kum Kee Corporate</t>
@@ -1729,10 +1785,14 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>yip-wai-chuen</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="n"/>
+          <t>Yip Wai Chuen | Employee Stories | Lee Kum Kee Corporate</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Yip Wai Chuen, Senior Production Manager at Lee Kum Kee. I have now become a mentor, who leads my less seasoned colleagues for their continuous learning a…</t>
+        </is>
+      </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
           <t>Yip Wai Chuen | Employee Stories | Lee Kum Kee Corporate</t>
@@ -1757,10 +1817,14 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>zhao-xiao-min</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="n"/>
+          <t>Zhao Xiao Min | Employee Stories | Lee Kum Kee Corporate</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Zhao Xiao Min, Senior HR Supervisor at Lee Kum Kee. Given my legal education, I am well aware of the importance of law-abiding business management which h…</t>
+        </is>
+      </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
           <t>Zhao Xiao Min | Employee Stories | Lee Kum Kee Corporate</t>
@@ -3029,10 +3093,14 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>adam-ho</t>
-        </is>
-      </c>
-      <c r="D91" s="2" t="n"/>
+          <t>何富贤 | 员工故事 | 李锦记企业</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>何富贤，信息科技经理，分享在李锦记的工作故事。「而很多时候，全靠与不同地区的团队一起讨论，发挥合作精神，我们才得以将问题解决。」</t>
+        </is>
+      </c>
       <c r="E91" s="4" t="inlineStr">
         <is>
           <t>何富贤 | 员工故事 | 李锦记企业</t>
@@ -3057,10 +3125,14 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>cheng-chiu-ming</t>
-        </is>
-      </c>
-      <c r="D92" s="2" t="n"/>
+          <t>郑照明（已退休） | 员工故事 | 李锦记企业</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>郑照明（已退休），生产经理，分享在李锦记的工作故事。「我认为企业文化是公司对员工必不可缺的指引，如果大家都能够实践集团的核心价值，将可令工作事半功倍。」</t>
+        </is>
+      </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
           <t>郑照明（已退休） | 员工故事 | 李锦记企业</t>
@@ -3085,10 +3157,14 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>cheng-wei-yan</t>
-        </is>
-      </c>
-      <c r="D93" s="2" t="n"/>
+          <t>程伟燕 | 员工故事 | 李锦记企业</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>程伟燕，助理经理，分享在李锦记的工作故事。「时至今日，我觉得最大的变化是我的管理职能比以前多，促使我懂得更全面地考虑各种问题。」</t>
+        </is>
+      </c>
       <c r="E93" s="4" t="inlineStr">
         <is>
           <t>程伟燕 | 员工故事 | 李锦记企业</t>
@@ -3113,10 +3189,14 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>gong-min</t>
-        </is>
-      </c>
-      <c r="D94" s="2" t="n"/>
+          <t>宫敏 | 员工故事 | 李锦记企业</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>宫敏，财务经理，分享在李锦记的工作故事。「作为一名负责税务的会计，我亦深深体会到公司『务实』、『诚信』的企业文化。」</t>
+        </is>
+      </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
           <t>宫敏 | 员工故事 | 李锦记企业</t>
@@ -3141,10 +3221,14 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>jiang-zhi</t>
-        </is>
-      </c>
-      <c r="D95" s="2" t="n"/>
+          <t>江智 | 员工故事 | 李锦记企业</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>江智，助理经理，分享在李锦记的工作故事。「我非常欣赏李锦记的企业文化，并以『务实』和『诚信』两个核心价值为自己在工作上的守则。」</t>
+        </is>
+      </c>
       <c r="E95" s="4" t="inlineStr">
         <is>
           <t>江智 | 员工故事 | 李锦记企业</t>
@@ -3169,10 +3253,14 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>lau-fung-ying-christine</t>
-        </is>
-      </c>
-      <c r="D96" s="2" t="n"/>
+          <t>刘凤英 | 员工故事 | 李锦记企业</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>刘凤英，高级业务发展经理，分享在李锦记的工作故事。「公司企业文化着重『换位思考』和『关注对方感受』，使我们在工作上能体察对方的需要。」</t>
+        </is>
+      </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
           <t>刘凤英 | 员工故事 | 李锦记企业</t>
@@ -3197,10 +3285,14 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>mark-butzke</t>
-        </is>
-      </c>
-      <c r="D97" s="2" t="n"/>
+          <t>Mark Butzke | 员工故事 | 李锦记企业</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>Mark Butzke，销售总监，分享在李锦记的工作故事。「一直以来，李锦记都为我提供所需的资源，助我发展事业。」</t>
+        </is>
+      </c>
       <c r="E97" s="4" t="inlineStr">
         <is>
           <t>Mark Butzke | 员工故事 | 李锦记企业</t>
@@ -3225,10 +3317,14 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>mauricio-olmedo</t>
-        </is>
-      </c>
-      <c r="D98" s="2" t="n"/>
+          <t>Mauricio Olmedo | 员工故事 | 李锦记企业</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>Mauricio Olmedo，生产经理，分享在李锦记的工作故事。「我不但获得了很多食品业丶生产流程和相关法规方面的知识，更学会了欣赏中菜！」</t>
+        </is>
+      </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
           <t>Mauricio Olmedo | 员工故事 | 李锦记企业</t>
@@ -3253,10 +3349,14 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>ng-seow-voon-miko</t>
-        </is>
-      </c>
-      <c r="D99" s="2" t="n"/>
+          <t>黄晓雯 | 员工故事 | 李锦记企业</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>黄晓雯，区域品类经理，分享在李锦记的工作故事。「虽然我加入李锦记的日子尚短，但我已经学会了很多，亦自觉变得更加成熟。」</t>
+        </is>
+      </c>
       <c r="E99" s="4" t="inlineStr">
         <is>
           <t>黄晓雯 | 员工故事 | 李锦记企业</t>
@@ -3281,10 +3381,14 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>ou-yang-tong</t>
-        </is>
-      </c>
-      <c r="D100" s="2" t="n"/>
+          <t>欧阳彤 | 员工故事 | 李锦记企业</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>欧阳彤，运营助理，分享在李锦记的工作故事。「尽管工作繁多、具有挑战，但却给了我一次又一次锻炼和成长的机会。」</t>
+        </is>
+      </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
           <t>欧阳彤 | 员工故事 | 李锦记企业</t>
@@ -3309,10 +3413,14 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>tony-mok</t>
-        </is>
-      </c>
-      <c r="D101" s="2" t="n"/>
+          <t>莫国栋 | 员工故事 | 李锦记企业</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>莫国栋，总经理 – 新会及黄埔厂，分享在李锦记的工作故事。「最初入职的时候，我只是制造部的见习主任，到今天，我管理接近3,000人的团队。」</t>
+        </is>
+      </c>
       <c r="E101" s="4" t="inlineStr">
         <is>
           <t>莫国栋 | 员工故事 | 李锦记企业</t>
@@ -3337,10 +3445,14 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>wei-gang</t>
-        </is>
-      </c>
-      <c r="D102" s="2" t="n"/>
+          <t>魏刚 | 员工故事 | 李锦记企业</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>魏刚，区域销售副总监-中大区，分享在李锦记的工作故事。「『100-1=0』是李锦记不断力求提升产品品质的企业文化，这种一丝不苟、追求完美的严谨态度，延伸到日常工作和管理中，令我们更能掌控结果，处事精益求精。」</t>
+        </is>
+      </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
           <t>魏刚 | 员工故事 | 李锦记企业</t>
@@ -3365,10 +3477,14 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>wen-wen</t>
-        </is>
-      </c>
-      <c r="D103" s="2" t="n"/>
+          <t>闻雯 | 员工故事 | 李锦记企业</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>闻雯，市场经理，分享在李锦记的工作故事。「我喜欢李锦记产品包装的经典设计，让人感觉质量有保障、很专业。」</t>
+        </is>
+      </c>
       <c r="E103" s="4" t="inlineStr">
         <is>
           <t>闻雯 | 员工故事 | 李锦记企业</t>
@@ -3393,10 +3509,14 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>wu-zhi-gang-jacky</t>
-        </is>
-      </c>
-      <c r="D104" s="2" t="n"/>
+          <t>吴志刚 | 员工故事 | 李锦记企业</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>吴志刚，运作总监，分享在李锦记的工作故事。「我认为持续学习很重要，加上团队内每一个人的力量，大家发挥各自的长处，才可事半功倍。」</t>
+        </is>
+      </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
           <t>吴志刚 | 员工故事 | 李锦记企业</t>
@@ -3421,10 +3541,14 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>yip-wai-chuen</t>
-        </is>
-      </c>
-      <c r="D105" s="2" t="n"/>
+          <t>叶伟全 | 员工故事 | 李锦记企业</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>叶伟全，高级生产经理，分享在李锦记的工作故事。「现在，我更像是一个师傅，带领着经验不足的同事从学习中迈向进步和成长。」</t>
+        </is>
+      </c>
       <c r="E105" s="4" t="inlineStr">
         <is>
           <t>叶伟全 | 员工故事 | 李锦记企业</t>
@@ -3449,10 +3573,14 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>zhao-xiao-min</t>
-        </is>
-      </c>
-      <c r="D106" s="2" t="n"/>
+          <t>赵晓敏 | 员工故事 | 李锦记企业</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>赵晓敏，高级人才资源主管，分享在李锦记的工作故事。「本着『永远创业精神』，我亦不断思考并调整自己的工作及沟通模式，努力学习新事物，工作日渐上轨道。」</t>
+        </is>
+      </c>
       <c r="E106" s="4" t="inlineStr">
         <is>
           <t>赵晓敏 | 员工故事 | 李锦记企业</t>
@@ -4637,10 +4765,14 @@
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>adam-ho</t>
-        </is>
-      </c>
-      <c r="D148" s="2" t="n"/>
+          <t>何富賢 | 員工故事 | 李錦記企業</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>何富賢，資訊科技經理，分享在李錦記的工作故事。「而很多時候，全靠與不同地區的團隊一起討論，發揮合作精神，我們才得以將問題解決。」</t>
+        </is>
+      </c>
       <c r="E148" s="4" t="inlineStr">
         <is>
           <t>何富賢 | 員工故事 | 李錦記企業</t>
@@ -4665,10 +4797,14 @@
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>cheng-chiu-ming</t>
-        </is>
-      </c>
-      <c r="D149" s="2" t="n"/>
+          <t>鄭照明（已退休） | 員工故事 | 李錦記企業</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>鄭照明（已退休），生產經理，分享在李錦記的工作故事。「我認為企業文化是公司對員工必不可缺的指引，如果大家都能夠實踐集團的核心價值，將可令工作事半功倍。」</t>
+        </is>
+      </c>
       <c r="E149" s="4" t="inlineStr">
         <is>
           <t>鄭照明（已退休） | 員工故事 | 李錦記企業</t>
@@ -4693,10 +4829,14 @@
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>cheng-wei-yan</t>
-        </is>
-      </c>
-      <c r="D150" s="2" t="n"/>
+          <t>程偉燕 | 員工故事 | 李錦記企業</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>程偉燕，助理經理，分享在李錦記的工作故事。「時至今日，我覺得最大的變化是我的管理職能比以前多，促使我懂得更全面地考慮各種問題。」</t>
+        </is>
+      </c>
       <c r="E150" s="4" t="inlineStr">
         <is>
           <t>程偉燕 | 員工故事 | 李錦記企業</t>
@@ -4721,10 +4861,14 @@
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>gong-min</t>
-        </is>
-      </c>
-      <c r="D151" s="2" t="n"/>
+          <t>宮敏 | 員工故事 | 李錦記企業</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>宮敏，財務經理，分享在李錦記的工作故事。「作為一名負責稅務的會計，我亦深深體會到公司『務實』、『誠信』的企業文化。」</t>
+        </is>
+      </c>
       <c r="E151" s="4" t="inlineStr">
         <is>
           <t>宮敏 | 員工故事 | 李錦記企業</t>
@@ -4749,10 +4893,14 @@
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>jiang-zhi</t>
-        </is>
-      </c>
-      <c r="D152" s="2" t="n"/>
+          <t>江智 | 員工故事 | 李錦記企業</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>江智，助理經理，分享在李錦記的工作故事。「我非常欣賞李錦記的企業文化，並以『務實』和『誠信』兩個核心價值為自己在工作上的守則。」</t>
+        </is>
+      </c>
       <c r="E152" s="4" t="inlineStr">
         <is>
           <t>江智 | 員工故事 | 李錦記企業</t>
@@ -4777,10 +4925,14 @@
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>lau-fung-ying-christine</t>
-        </is>
-      </c>
-      <c r="D153" s="2" t="n"/>
+          <t>劉鳳英 | 員工故事 | 李錦記企業</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>劉鳳英，高級業務發展經理，分享在李錦記的工作故事。「公司企業文化著重『換位思考』和『關注對方感受』，使我們在工作上能體察對方的需要。」</t>
+        </is>
+      </c>
       <c r="E153" s="4" t="inlineStr">
         <is>
           <t>劉鳳英 | 員工故事 | 李錦記企業</t>
@@ -4805,10 +4957,14 @@
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>mark-butzke</t>
-        </is>
-      </c>
-      <c r="D154" s="2" t="n"/>
+          <t>Mark Butzke | 員工故事 | 李錦記企業</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>Mark Butzke，銷售總監，分享在李錦記的工作故事。「一直以來，李錦記都為我提供所需的資源，助我發展事業。」</t>
+        </is>
+      </c>
       <c r="E154" s="4" t="inlineStr">
         <is>
           <t>Mark Butzke | 員工故事 | 李錦記企業</t>
@@ -4833,10 +4989,14 @@
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>mauricio-olmedo</t>
-        </is>
-      </c>
-      <c r="D155" s="2" t="n"/>
+          <t>Mauricio Olmedo | 員工故事 | 李錦記企業</t>
+        </is>
+      </c>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>Mauricio Olmedo，生產經理，分享在李錦記的工作故事。「我不但獲得了很多食品業、生產流程和相關法規方面的知識，更學會了欣賞中菜！」</t>
+        </is>
+      </c>
       <c r="E155" s="4" t="inlineStr">
         <is>
           <t>Mauricio Olmedo | 員工故事 | 李錦記企業</t>
@@ -4861,10 +5021,14 @@
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>ng-seow-voon-miko</t>
-        </is>
-      </c>
-      <c r="D156" s="2" t="n"/>
+          <t>黃曉雯 | 員工故事 | 李錦記企業</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>黃曉雯，區域品類經理，分享在李錦記的工作故事。「雖然我加入李錦記的日子尚短，但我已經學會了很多，亦自覺變得更加成熟。」</t>
+        </is>
+      </c>
       <c r="E156" s="4" t="inlineStr">
         <is>
           <t>黃曉雯 | 員工故事 | 李錦記企業</t>
@@ -4889,10 +5053,14 @@
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>ou-yang-tong</t>
-        </is>
-      </c>
-      <c r="D157" s="2" t="n"/>
+          <t>歐陽彤 | 員工故事 | 李錦記企業</t>
+        </is>
+      </c>
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>歐陽彤，運營助理，分享在李錦記的工作故事。「儘管工作繁多、具有挑戰，但卻給了我一次又一次鍛煉和成長的機會。」</t>
+        </is>
+      </c>
       <c r="E157" s="4" t="inlineStr">
         <is>
           <t>歐陽彤 | 員工故事 | 李錦記企業</t>
@@ -4917,10 +5085,14 @@
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>tony-mok</t>
-        </is>
-      </c>
-      <c r="D158" s="2" t="n"/>
+          <t>莫國棟 | 員工故事 | 李錦記企業</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>莫國棟，總經理 – 新會及黃埔廠，分享在李錦記的工作故事。「最初入職的時候，我只是製造部的見習主任，到今天，我管理接近3,000人的團隊。」</t>
+        </is>
+      </c>
       <c r="E158" s="4" t="inlineStr">
         <is>
           <t>莫國棟 | 員工故事 | 李錦記企業</t>
@@ -4945,10 +5117,14 @@
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>wei-gang</t>
-        </is>
-      </c>
-      <c r="D159" s="2" t="n"/>
+          <t>魏剛 | 員工故事 | 李錦記企業</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>魏剛，區域銷售副總監 - 中大區，分享在李錦記的工作故事。「『100-1=0』是李錦記不斷力求提升產品品質的企業文化，這種一絲不苟、追求完美的嚴謹態度，延伸到日常工作和管理中，令我們更能掌控結果，處事精益求精。」</t>
+        </is>
+      </c>
       <c r="E159" s="4" t="inlineStr">
         <is>
           <t>魏剛 | 員工故事 | 李錦記企業</t>
@@ -4973,10 +5149,14 @@
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>wen-wen</t>
-        </is>
-      </c>
-      <c r="D160" s="2" t="n"/>
+          <t>聞雯 | 員工故事 | 李錦記企業</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>聞雯，市場經理，分享在李錦記的工作故事。「我喜歡李錦記產品包裝的經典設計，讓人感覺品質有保障、很專業。」</t>
+        </is>
+      </c>
       <c r="E160" s="4" t="inlineStr">
         <is>
           <t>聞雯 | 員工故事 | 李錦記企業</t>
@@ -5001,10 +5181,14 @@
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>wu-zhi-gang-jacky</t>
-        </is>
-      </c>
-      <c r="D161" s="2" t="n"/>
+          <t>吳志剛 | 員工故事 | 李錦記企業</t>
+        </is>
+      </c>
+      <c r="D161" s="2" t="inlineStr">
+        <is>
+          <t>吳志剛，運作總監，分享在李錦記的工作故事。「我認為持續學習很重要，加上團隊內每一個人的力量，大家發揮各自的長處，才可事半功倍。」</t>
+        </is>
+      </c>
       <c r="E161" s="4" t="inlineStr">
         <is>
           <t>吳志剛 | 員工故事 | 李錦記企業</t>
@@ -5029,10 +5213,14 @@
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>yip-wai-chuen</t>
-        </is>
-      </c>
-      <c r="D162" s="2" t="n"/>
+          <t>葉偉全 | 員工故事 | 李錦記企業</t>
+        </is>
+      </c>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>葉偉全，高級生產經理，分享在李錦記的工作故事。「現在，我更像是一個師傅，帶領著經驗不足的同事從學習中邁向進步和成長。」</t>
+        </is>
+      </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
           <t>葉偉全 | 員工故事 | 李錦記企業</t>
@@ -5057,10 +5245,14 @@
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>zhao-xiao-min</t>
-        </is>
-      </c>
-      <c r="D163" s="2" t="n"/>
+          <t>趙曉敏 | 員工故事 | 李錦記企業</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>趙曉敏，高級人才資源主管，分享在李錦記的工作故事。「本着『永遠創業精神』，我亦不斷思考並調整自己的工作及溝通模式，努力學習新事物，工作日漸上軌道。」</t>
+        </is>
+      </c>
       <c r="E163" s="4" t="inlineStr">
         <is>
           <t>趙曉敏 | 員工故事 | 李錦記企業</t>

</xml_diff>